<commit_message>
Add multi-entity EP sample and refresh the SIT template.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Template/SIT Template.xlsx
+++ b/Template/SIT Template.xlsx
@@ -7,7 +7,7 @@
     <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
-    <sheet name="08-09-26 (2)" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2 (2)" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -27,9 +27,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="30">
-  <si>
-    <t>General Uganda | SIT -Module-wise Daily Status</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="33">
+  <si>
+    <t xml:space="preserve">General Uganda | SIT (QA) </t>
   </si>
   <si>
     <t>Lead Champion</t>
@@ -65,13 +65,22 @@
     <t>Fixed Assets Management</t>
   </si>
   <si>
+    <t>Procurement</t>
+  </si>
+  <si>
+    <t>Cash and Bank Management</t>
+  </si>
+  <si>
+    <t>General Ledger</t>
+  </si>
+  <si>
     <t xml:space="preserve">Execution Rate </t>
   </si>
   <si>
     <t>Overall Pass Rate</t>
   </si>
   <si>
-    <t>Life Uganda | SIT -Module-wise Daily Status</t>
+    <t>Life Uganda | SIT (QA)</t>
   </si>
   <si>
     <t>Bernard Towett</t>
@@ -83,7 +92,7 @@
     <t>Intergations (ILMS)</t>
   </si>
   <si>
-    <t>General Tanzania  | SIT -Module-wise Daily Status</t>
+    <t>General Tanzania  | SIT (QA)</t>
   </si>
   <si>
     <t>Dennis Thea</t>
@@ -464,13 +473,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF5B9BD5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -685,7 +694,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -725,9 +734,33 @@
       <top style="thin">
         <color auto="1"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -902,7 +935,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -914,34 +947,34 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="21" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="22" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="21" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1026,7 +1059,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1072,58 +1105,76 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1138,52 +1189,52 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1195,46 +1246,40 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1243,10 +1288,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1774,7 +1819,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J55"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.4444444444444" style="1" customWidth="1"/>
@@ -1786,7 +1831,7 @@
     <col min="7" max="7" width="11" style="1" customWidth="1"/>
     <col min="8" max="8" width="13.2222222222222" style="1" customWidth="1"/>
     <col min="9" max="9" width="7.25" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.88888888888889" style="1" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="8.88888888888889" style="1" customWidth="1"/>
     <col min="11" max="11" width="8.88888888888889" style="1"/>
     <col min="12" max="12" width="12.8888888888889" style="1"/>
     <col min="13" max="13" width="27.8888888888889" style="1" customWidth="1"/>
@@ -1850,707 +1895,889 @@
       <c r="G4" s="16"/>
       <c r="H4" s="16"/>
       <c r="I4" s="17">
-        <f>SUM(D4:H4)</f>
+        <f t="shared" ref="I4:I7" si="0">SUM(D4:H4)</f>
         <v>0</v>
       </c>
       <c r="J4" s="18" t="e">
-        <f>D4/(I4-F4)</f>
+        <f t="shared" ref="J4:J8" si="1">D4/(I4-F4)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
-      <c r="B5" s="19"/>
-      <c r="C5" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="20">
-        <f t="shared" ref="D5:I5" si="0">SUM(D4:D4)</f>
-        <v>0</v>
-      </c>
-      <c r="E5" s="21">
+      <c r="A5" s="19"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="17">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F5" s="22">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G5" s="23">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H5" s="24">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I5" s="25">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J5" s="26" t="e">
-        <f>D5/(I5-F5)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="6" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="D6" s="27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="28" t="e">
-        <f>(D5+E5)/(I5-F5)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H6" s="28"/>
-      <c r="I6" s="28"/>
-    </row>
-    <row r="7" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="D7" s="29" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="29"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="30" t="e">
-        <f>D5/(I5-F5)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-    </row>
-    <row r="10" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B10" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" s="1" customFormat="1" ht="18" customHeight="1" spans="1:10">
-      <c r="B11" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B12" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="H12" s="16"/>
-      <c r="I12" s="17">
-        <f>SUM(D12:H12)</f>
-        <v>0</v>
-      </c>
-      <c r="J12" s="26" t="e">
-        <f t="shared" ref="J12:J14" si="1">D12/(I12-F12)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="13" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B13" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="H13" s="16"/>
-      <c r="I13" s="17">
-        <f>SUM(D13:H13)</f>
-        <v>0</v>
-      </c>
-      <c r="J13" s="26" t="e">
+      <c r="J5" s="21" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="14" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B14" s="32"/>
-      <c r="C14" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="D14" s="20">
-        <f t="shared" ref="D14:I14" si="2">SUM(D12:D13)</f>
-        <v>0</v>
-      </c>
-      <c r="E14" s="21">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F14" s="22">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G14" s="23">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="24">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="25">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J14" s="26" t="e">
+    <row r="6" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
+      <c r="A6" s="19"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="16"/>
+      <c r="H6" s="16"/>
+      <c r="I6" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="21" t="e">
         <f t="shared" si="1"/>
         <v>#DIV/0!</v>
       </c>
     </row>
+    <row r="7" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
+      <c r="A7" s="19"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16"/>
+      <c r="H7" s="16"/>
+      <c r="I7" s="17">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="18" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="8" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
+      <c r="B8" s="23"/>
+      <c r="C8" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="25">
+        <f t="shared" ref="D8:I8" si="2">SUM(D4:D7)</f>
+        <v>0</v>
+      </c>
+      <c r="E8" s="26">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="F8" s="27">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="28">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="H8" s="29">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="I8" s="30">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J8" s="31" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="9" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="D9" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="33" t="e">
+        <f>(D8+E8)/(I8-F8)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+    </row>
+    <row r="10" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="D10" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="35" t="e">
+        <f>D8/(I8-F8)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H10" s="35"/>
+      <c r="I10" s="35"/>
+    </row>
+    <row r="13" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="B13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" s="1" customFormat="1" ht="18" customHeight="1" spans="1:10">
+      <c r="B14" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I14" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
     <row r="15" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="D15" s="27" t="s">
+      <c r="B15" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="17">
+        <f t="shared" ref="I15:I19" si="3">SUM(D15:H15)</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="21" t="e">
+        <f t="shared" ref="J15:J20" si="4">D15/(I15-F15)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="16" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="B16" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J16" s="37" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B17" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="28" t="e">
-        <f>(D14+E14)/(I14-F14)</f>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J17" s="18" t="e">
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-    </row>
-    <row r="16" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="D16" s="29" t="s">
+    </row>
+    <row r="18" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B18" s="20"/>
+      <c r="C18" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="30" t="e">
-        <f>D14/(I14-F14)</f>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="21" t="e">
+        <f t="shared" si="4"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-    </row>
-    <row r="18" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A18" s="1"/>
-      <c r="B18" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-    </row>
-    <row r="19" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A19" s="1"/>
-      <c r="B19" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I19" s="11" t="s">
+    </row>
+    <row r="19" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B19" s="22"/>
+      <c r="C19" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="17">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="18" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B20" s="38"/>
+      <c r="C20" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="J19" s="12" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="20" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A20" s="1"/>
-      <c r="B20" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="17">
-        <f>SUM(D20:H20)</f>
-        <v>0</v>
-      </c>
-      <c r="J20" s="26" t="e">
+      <c r="D20" s="25">
+        <f t="shared" ref="D20:I20" si="5">SUM(D15:D19)</f>
+        <v>0</v>
+      </c>
+      <c r="E20" s="26">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="F20" s="27">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="28">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H20" s="29">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="30">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="31" t="e">
+        <f t="shared" si="4"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="D21" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="33" t="e">
+        <f>(D20+E20)/(I20-F20)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H21" s="33"/>
+      <c r="I21" s="33"/>
+    </row>
+    <row r="22" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="D22" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="34"/>
+      <c r="F22" s="34"/>
+      <c r="G22" s="35" t="e">
         <f>D20/(I20-F20)</f>
         <v>#DIV/0!</v>
       </c>
-    </row>
-    <row r="21" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A21" s="1"/>
-      <c r="B21" s="32"/>
-      <c r="C21" s="14" t="s">
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+    </row>
+    <row r="24" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B25" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I25" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D21" s="20">
-        <f t="shared" ref="D21:I21" si="3">SUM(D20:D20)</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="21">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F21" s="22">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="G21" s="23">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="H21" s="24">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="I21" s="25">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J21" s="26" t="e">
-        <f>D21/(I21-F21)</f>
+      <c r="J25" s="12" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="26" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B26" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="17">
+        <f t="shared" ref="I26:I29" si="6">SUM(D26:H26)</f>
+        <v>0</v>
+      </c>
+      <c r="J26" s="18" t="e">
+        <f t="shared" ref="J26:J30" si="7">D26/(I26-F26)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="22" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="27" t="s">
+    <row r="27" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B27" s="20"/>
+      <c r="C27" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="28" t="e">
-        <f>(D21+E21)/(I21-F21)</f>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J27" s="18" t="e">
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H22" s="28"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="1"/>
-    </row>
-    <row r="23" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="29" t="s">
+    </row>
+    <row r="28" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B28" s="20"/>
+      <c r="C28" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="29"/>
-      <c r="F23" s="29"/>
-      <c r="G23" s="30" t="e">
-        <f>D21/(I21-F21)</f>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="16"/>
+      <c r="H28" s="16"/>
+      <c r="I28" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J28" s="18" t="e">
+        <f t="shared" si="7"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="1"/>
-    </row>
-    <row r="24" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="34"/>
-      <c r="I24" s="35"/>
-      <c r="J24" s="1"/>
-    </row>
-    <row r="25" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="A25" s="1">
-        <f>80+84</f>
+    </row>
+    <row r="29" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B29" s="22"/>
+      <c r="C29" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J29" s="18" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="30" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B30" s="38"/>
+      <c r="C30" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D30" s="25">
+        <f t="shared" ref="D30:H30" si="8">SUM(D26:D29)</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="26">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="F30" s="27">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="G30" s="28">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="H30" s="29">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="I30" s="30">
+        <f>SUM(I26:I28)</f>
+        <v>0</v>
+      </c>
+      <c r="J30" s="31" t="e">
+        <f t="shared" si="7"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="D31" s="32" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="33" t="e">
+        <f>(D30+E30)/(I30-F30)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H31" s="33"/>
+      <c r="I31" s="33"/>
+    </row>
+    <row r="32" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="D32" s="34" t="s">
+        <v>16</v>
+      </c>
+      <c r="E32" s="34"/>
+      <c r="F32" s="34"/>
+      <c r="G32" s="35" t="e">
+        <f>D30/(I30-F30)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H32" s="35"/>
+      <c r="I32" s="35"/>
+    </row>
+    <row r="33" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="D33" s="39"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="40"/>
+      <c r="H33" s="40"/>
+      <c r="I33" s="41"/>
+    </row>
+    <row r="34" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="A34" s="1">
         <v>164</v>
       </c>
-      <c r="B25" s="36"/>
-      <c r="C25" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="37"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="37"/>
-      <c r="H25" s="37"/>
-    </row>
-    <row r="26" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="C26" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D26" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E26" s="39" t="s">
+      <c r="B34" s="42"/>
+      <c r="C34" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="40" t="s">
+      <c r="D34" s="43"/>
+      <c r="E34" s="43"/>
+      <c r="F34" s="43"/>
+      <c r="G34" s="43"/>
+      <c r="H34" s="43"/>
+    </row>
+    <row r="35" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C35" s="44" t="s">
         <v>24</v>
       </c>
-      <c r="G26" s="41" t="s">
+      <c r="D35" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="H26" s="42" t="s">
+      <c r="E35" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F35" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="G35" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="H35" s="48" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="27" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="C27" s="15" t="s">
+    <row r="36" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C36" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="44"/>
-      <c r="G27" s="44"/>
-      <c r="H27" s="45">
-        <f>SUM(D27:G27)</f>
-        <v>0</v>
-      </c>
-      <c r="I27" s="46"/>
-    </row>
-    <row r="28" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="C28" s="38" t="s">
+      <c r="D36" s="49"/>
+      <c r="E36" s="49"/>
+      <c r="F36" s="50"/>
+      <c r="G36" s="50"/>
+      <c r="H36" s="51">
+        <f>SUM(D36:G36)</f>
+        <v>0</v>
+      </c>
+      <c r="I36" s="52"/>
+    </row>
+    <row r="37" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C37" s="44" t="s">
         <v>8</v>
       </c>
-      <c r="D28" s="47">
-        <f t="shared" ref="D28:H28" si="4">SUM(D27:D27)</f>
-        <v>0</v>
-      </c>
-      <c r="E28" s="47">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="F28" s="48">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="G28" s="48">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="H28" s="49">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I28" s="46"/>
-    </row>
-    <row r="29" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="C29" s="50"/>
-      <c r="D29" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="E29" s="51"/>
-      <c r="F29" s="52" t="e">
-        <f>(D28+E28)/H28</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G29" s="52"/>
-      <c r="H29" s="53"/>
-      <c r="I29" s="46"/>
-    </row>
-    <row r="30" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B30" s="54"/>
-      <c r="C30" s="55"/>
-      <c r="D30" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="E30" s="57"/>
-      <c r="F30" s="52" t="e">
-        <f>(D28+E28+F28)/H28</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G30" s="52"/>
-      <c r="H30" s="58"/>
-      <c r="I30" s="46"/>
-    </row>
-    <row r="31" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B31" s="54"/>
-      <c r="C31" s="54"/>
-      <c r="D31" s="59"/>
-      <c r="E31" s="59"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="61"/>
-      <c r="I31" s="46"/>
-    </row>
-    <row r="32" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B32" s="36"/>
-      <c r="C32" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="D32" s="37"/>
-      <c r="E32" s="37"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="37"/>
-      <c r="H32" s="37"/>
-      <c r="I32" s="46"/>
-    </row>
-    <row r="33" s="1" customFormat="1" ht="15.6" spans="2:9">
-      <c r="B33" s="62"/>
-      <c r="C33" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D33" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E33" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F33" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="G33" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="H33" s="42" t="s">
-        <v>8</v>
-      </c>
-      <c r="I33" s="46"/>
-    </row>
-    <row r="34" s="1" customFormat="1" ht="15.6" spans="2:9">
-      <c r="B34" s="62"/>
-      <c r="C34" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="63"/>
-      <c r="E34" s="63"/>
-      <c r="F34" s="64"/>
-      <c r="G34" s="64"/>
-      <c r="H34" s="65">
-        <f>SUM(D34:G34)</f>
-        <v>0</v>
-      </c>
-      <c r="I34" s="46"/>
-    </row>
-    <row r="35" s="1" customFormat="1" ht="15.6" spans="2:9">
-      <c r="B35" s="62"/>
-      <c r="C35" s="38" t="s">
-        <v>8</v>
-      </c>
-      <c r="D35" s="66">
-        <f t="shared" ref="D35:H35" si="5">SUM(D34:D34)</f>
-        <v>0</v>
-      </c>
-      <c r="E35" s="66">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F35" s="67">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="G35" s="68">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="H35" s="69">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" s="1" customFormat="1" ht="15.6" spans="2:9">
-      <c r="B36" s="70"/>
-      <c r="C36" s="54"/>
-      <c r="D36" s="51" t="s">
-        <v>26</v>
-      </c>
-      <c r="E36" s="51"/>
-      <c r="F36" s="52" t="e">
-        <f>(D35+E35)/H35</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G36" s="52"/>
-      <c r="H36" s="71"/>
-    </row>
-    <row r="37" s="1" customFormat="1" ht="15.6" spans="2:9">
-      <c r="B37" s="70"/>
-      <c r="C37" s="54"/>
-      <c r="D37" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="E37" s="57"/>
-      <c r="F37" s="72" t="e">
-        <f>(D35+E35+F35)/H35</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G37" s="73"/>
-      <c r="H37" s="71"/>
-    </row>
-    <row r="39" ht="15.6" spans="2:9">
-      <c r="C39" s="37" t="s">
+      <c r="D37" s="53">
+        <f t="shared" ref="D37:G37" si="9">SUM(D36:D36)</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="53">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="F37" s="54">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="G37" s="54">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+      <c r="H37" s="55">
+        <f>SUM(D37:G37)</f>
+        <v>0</v>
+      </c>
+      <c r="I37" s="52"/>
+    </row>
+    <row r="38" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C38" s="56"/>
+      <c r="D38" s="57" t="s">
         <v>29</v>
       </c>
-      <c r="D39" s="37"/>
-      <c r="E39" s="37"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="37"/>
-      <c r="H39" s="37"/>
-    </row>
-    <row r="40" ht="15.6" spans="2:9">
-      <c r="C40" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="D40" s="29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E40" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="F40" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="G40" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="H40" s="42" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="41" ht="15.6" spans="2:9">
-      <c r="C41" s="15" t="s">
-        <v>11</v>
+      <c r="E38" s="57"/>
+      <c r="F38" s="58">
+        <v>0</v>
+      </c>
+      <c r="G38" s="58"/>
+      <c r="H38" s="59"/>
+      <c r="I38" s="52"/>
+    </row>
+    <row r="39" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B39" s="60"/>
+      <c r="C39" s="61"/>
+      <c r="D39" s="62" t="s">
+        <v>30</v>
+      </c>
+      <c r="E39" s="63"/>
+      <c r="F39" s="58">
+        <v>0</v>
+      </c>
+      <c r="G39" s="58"/>
+      <c r="H39" s="52"/>
+      <c r="I39" s="52"/>
+    </row>
+    <row r="40" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B40" s="60"/>
+      <c r="C40" s="60"/>
+      <c r="D40" s="64"/>
+      <c r="E40" s="64"/>
+      <c r="F40" s="65"/>
+      <c r="G40" s="66"/>
+      <c r="I40" s="52"/>
+    </row>
+    <row r="41" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B41" s="42"/>
+      <c r="C41" s="43" t="s">
+        <v>31</v>
       </c>
       <c r="D41" s="43"/>
       <c r="E41" s="43"/>
-      <c r="F41" s="44"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="45">
-        <f>SUM(D41:G41)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" ht="15.6" spans="2:9">
-      <c r="C42" s="38" t="s">
+      <c r="F41" s="43"/>
+      <c r="G41" s="43"/>
+      <c r="H41" s="43"/>
+      <c r="I41" s="52"/>
+    </row>
+    <row r="42" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B42" s="39"/>
+      <c r="C42" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="D42" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E42" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F42" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="G42" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="H42" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="D42" s="47">
-        <f t="shared" ref="D42:H42" si="6">SUM(D41:D41)</f>
-        <v>0</v>
-      </c>
-      <c r="E42" s="47">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="F42" s="48">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="G42" s="48">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="H42" s="49">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" s="1" customFormat="1" ht="16" customHeight="1" spans="2:9">
-      <c r="C43" s="50"/>
-      <c r="D43" s="51" t="s">
+      <c r="I42" s="52"/>
+    </row>
+    <row r="43" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B43" s="39"/>
+      <c r="C43" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="67"/>
+      <c r="E43" s="67"/>
+      <c r="F43" s="68"/>
+      <c r="G43" s="68"/>
+      <c r="H43" s="69">
+        <f>SUM(D43:G43)</f>
+        <v>0</v>
+      </c>
+      <c r="I43" s="52"/>
+    </row>
+    <row r="44" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B44" s="39"/>
+      <c r="C44" s="44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D44" s="70">
+        <f>SUM(D43:D43)</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="70">
+        <f>SUM(E43:E43)</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="71">
+        <f>SUM(F43:F43)</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="72">
+        <f>SUM(G43:G43)</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="73">
+        <f>SUM(D44:G44)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B45" s="74"/>
+      <c r="C45" s="60"/>
+      <c r="D45" s="57" t="s">
+        <v>29</v>
+      </c>
+      <c r="E45" s="57"/>
+      <c r="F45" s="58">
+        <v>0</v>
+      </c>
+      <c r="G45" s="58"/>
+      <c r="H45" s="75"/>
+    </row>
+    <row r="46" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B46" s="74"/>
+      <c r="C46" s="60"/>
+      <c r="D46" s="62" t="s">
+        <v>30</v>
+      </c>
+      <c r="E46" s="63"/>
+      <c r="F46" s="76">
+        <v>0</v>
+      </c>
+      <c r="G46" s="77"/>
+      <c r="H46" s="75"/>
+    </row>
+    <row r="48" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C48" s="43" t="s">
+        <v>32</v>
+      </c>
+      <c r="D48" s="43"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="43"/>
+    </row>
+    <row r="49" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C49" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="D49" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E49" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="E43" s="51"/>
-      <c r="F43" s="52" t="e">
-        <f>(D42+E42)/H42</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G43" s="52"/>
-      <c r="H43" s="53"/>
-    </row>
-    <row r="44" ht="15.6" spans="2:9">
-      <c r="C44" s="55"/>
-      <c r="D44" s="56" t="s">
+      <c r="F49" s="46" t="s">
         <v>27</v>
       </c>
-      <c r="E44" s="57"/>
-      <c r="F44" s="52" t="e">
-        <f>(D42+E42+F42)/H42</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="G44" s="52"/>
-      <c r="H44" s="58"/>
+      <c r="G49" s="47" t="s">
+        <v>28</v>
+      </c>
+      <c r="H49" s="48" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C50" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" s="49"/>
+      <c r="E50" s="49"/>
+      <c r="F50" s="50"/>
+      <c r="G50" s="50"/>
+      <c r="H50" s="51">
+        <f>SUM(D50:G50)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C51" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D51" s="49"/>
+      <c r="E51" s="49"/>
+      <c r="F51" s="50"/>
+      <c r="G51" s="50"/>
+      <c r="H51" s="51">
+        <f>SUM(D51:G51)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C52" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" s="49"/>
+      <c r="E52" s="49"/>
+      <c r="F52" s="50"/>
+      <c r="G52" s="50"/>
+      <c r="H52" s="51">
+        <f>SUM(D52:G52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C53" s="44" t="s">
+        <v>8</v>
+      </c>
+      <c r="D53" s="53">
+        <f>SUM(D50:D52)</f>
+        <v>0</v>
+      </c>
+      <c r="E53" s="53">
+        <f>SUM(E50:E52)</f>
+        <v>0</v>
+      </c>
+      <c r="F53" s="54">
+        <f>SUM(F50:F52)</f>
+        <v>0</v>
+      </c>
+      <c r="G53" s="54">
+        <f>SUM(G50:G52)</f>
+        <v>0</v>
+      </c>
+      <c r="H53" s="55">
+        <f>SUM(H50:H52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" s="1" customFormat="1" ht="16" customHeight="1" spans="3:8">
+      <c r="C54" s="56"/>
+      <c r="D54" s="57" t="s">
+        <v>29</v>
+      </c>
+      <c r="E54" s="57"/>
+      <c r="F54" s="58">
+        <v>0</v>
+      </c>
+      <c r="G54" s="58"/>
+      <c r="H54" s="59"/>
+    </row>
+    <row r="55" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C55" s="61"/>
+      <c r="D55" s="62" t="s">
+        <v>30</v>
+      </c>
+      <c r="E55" s="63"/>
+      <c r="F55" s="58">
+        <v>0</v>
+      </c>
+      <c r="G55" s="58"/>
+      <c r="H55" s="52"/>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="33">
     <mergeCell ref="B2:J2"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="B10:J10"/>
-    <mergeCell ref="D15:F15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="D16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="B18:J18"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="B13:J13"/>
+    <mergeCell ref="D21:F21"/>
+    <mergeCell ref="G21:I21"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="G22:I22"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="B24:J24"/>
+    <mergeCell ref="D31:F31"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="D32:F32"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="C48:H48"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B26:B29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Enable per-project defect Entity columns and Sprint 3 sprint filtering in Reporter.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Template/SIT Template.xlsx
+++ b/Template/SIT Template.xlsx
@@ -27,9 +27,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="33">
-  <si>
-    <t xml:space="preserve">General Uganda | SIT (QA) </t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="35">
+  <si>
+    <t>General Uganda | SIT (QA) -Module-wise Daily Status</t>
   </si>
   <si>
     <t>Lead Champion</t>
@@ -71,6 +71,12 @@
     <t>Cash and Bank Management</t>
   </si>
   <si>
+    <t>Mambo Muia</t>
+  </si>
+  <si>
+    <t>Intergations (Footprint)</t>
+  </si>
+  <si>
     <t>General Ledger</t>
   </si>
   <si>
@@ -80,7 +86,7 @@
     <t>Overall Pass Rate</t>
   </si>
   <si>
-    <t>Life Uganda | SIT (QA)</t>
+    <t>Life Uganda | SIT (QA) -Module-wise Daily Status</t>
   </si>
   <si>
     <t>Bernard Towett</t>
@@ -92,7 +98,7 @@
     <t>Intergations (ILMS)</t>
   </si>
   <si>
-    <t>General Tanzania  | SIT (QA)</t>
+    <t>General Tanzania  | SIT (QA) -Module-wise Daily Status</t>
   </si>
   <si>
     <t>Dennis Thea</t>
@@ -398,7 +404,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="50">
+  <fills count="49">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -546,12 +552,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -734,7 +734,9 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -747,9 +749,7 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -986,80 +986,80 @@
     <xf numFmtId="0" fontId="32" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="43" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="44" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="45" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="46" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="34" fillId="47" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="49" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="48" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="78">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1105,76 +1105,70 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="3" fillId="13" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="3" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="11" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1189,52 +1183,52 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1246,10 +1240,10 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1261,25 +1255,25 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1819,7 +1813,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="17.4444444444444" style="1" customWidth="1"/>
@@ -1895,17 +1889,17 @@
       <c r="G4" s="16"/>
       <c r="H4" s="16"/>
       <c r="I4" s="17">
-        <f t="shared" ref="I4:I7" si="0">SUM(D4:H4)</f>
+        <f>SUM(D4:H4)</f>
         <v>0</v>
       </c>
       <c r="J4" s="18" t="e">
-        <f t="shared" ref="J4:J8" si="1">D4/(I4-F4)</f>
+        <f>D4/(I4-F4)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
       <c r="A5" s="19"/>
-      <c r="B5" s="20"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="15" t="s">
         <v>12</v>
       </c>
@@ -1915,17 +1909,17 @@
       <c r="G5" s="16"/>
       <c r="H5" s="16"/>
       <c r="I5" s="17">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J5" s="21" t="e">
-        <f t="shared" si="1"/>
+        <f>SUM(D5:H5)</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="20" t="e">
+        <f>D5/(I5-F5)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
       <c r="A6" s="19"/>
-      <c r="B6" s="20"/>
+      <c r="B6" s="14"/>
       <c r="C6" s="15" t="s">
         <v>13</v>
       </c>
@@ -1935,163 +1929,160 @@
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
       <c r="I6" s="17">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J6" s="21" t="e">
-        <f t="shared" si="1"/>
+        <f>SUM(D6:H6)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="20" t="e">
+        <f>D6/(I6-F6)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
       <c r="A7" s="19"/>
-      <c r="B7" s="22"/>
+      <c r="B7" s="14" t="s">
+        <v>14</v>
+      </c>
       <c r="C7" s="15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
-      <c r="I7" s="17">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J7" s="18" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="I7" s="17"/>
+      <c r="J7" s="20"/>
     </row>
     <row r="8" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
-      <c r="B8" s="23"/>
-      <c r="C8" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="25">
-        <f t="shared" ref="D8:I8" si="2">SUM(D4:D7)</f>
-        <v>0</v>
-      </c>
-      <c r="E8" s="26">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F8" s="27">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="28">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H8" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="30">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J8" s="31" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="D9" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="33" t="e">
-        <f>(D8+E8)/(I8-F8)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-    </row>
-    <row r="10" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="D10" s="34" t="s">
+      <c r="A8" s="19"/>
+      <c r="B8" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="35" t="e">
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="16"/>
+      <c r="I8" s="17">
+        <f>SUM(D8:H8)</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="18" t="e">
         <f>D8/(I8-F8)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H10" s="35"/>
-      <c r="I10" s="35"/>
-    </row>
-    <row r="13" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B13" s="2" t="s">
+    </row>
+    <row r="9" s="1" customFormat="1" ht="15.6" customHeight="1" spans="1:10">
+      <c r="B9" s="22"/>
+      <c r="C9" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="23">
+        <f t="shared" ref="D9:I9" si="0">SUM(D4:D8)</f>
+        <v>0</v>
+      </c>
+      <c r="E9" s="24">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="F9" s="25">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G9" s="26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="H9" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I9" s="28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J9" s="29" t="e">
+        <f>D9/(I9-F9)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="10" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="D10" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-    </row>
-    <row r="14" s="1" customFormat="1" ht="18" customHeight="1" spans="1:10">
-      <c r="B14" s="4" t="s">
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="31" t="e">
+        <f>(D9+E9)/(I9-F9)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+    </row>
+    <row r="11" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="D11" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="29" t="e">
+        <f>D9/(I9-F9)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
+    </row>
+    <row r="14" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="B14" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" s="1" customFormat="1" ht="18" customHeight="1" spans="1:10">
+      <c r="B15" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D15" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E15" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F15" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G14" s="9" t="s">
+      <c r="G15" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H14" s="10" t="s">
+      <c r="H15" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="I15" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="J14" s="12" t="s">
+      <c r="J15" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="15" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B15" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="15" t="s">
+    <row r="16" s="1" customFormat="1" ht="15.6" spans="1:10">
+      <c r="B16" s="14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="15" t="s">
         <v>11</v>
-      </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
-      <c r="H15" s="16"/>
-      <c r="I15" s="17">
-        <f t="shared" ref="I15:I19" si="3">SUM(D15:H15)</f>
-        <v>0</v>
-      </c>
-      <c r="J15" s="21" t="e">
-        <f t="shared" ref="J15:J20" si="4">D15/(I15-F15)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="16" s="1" customFormat="1" ht="15.6" spans="1:10">
-      <c r="B16" s="36" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>20</v>
       </c>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -2099,20 +2090,20 @@
       <c r="G16" s="16"/>
       <c r="H16" s="16"/>
       <c r="I16" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J16" s="37" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="I16:I20" si="1">SUM(D16:H16)</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="20" t="e">
+        <f t="shared" ref="J16:J21" si="2">D16/(I16-F16)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="1" ht="15.6" spans="2:10">
       <c r="B17" s="14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
@@ -2120,18 +2111,20 @@
       <c r="G17" s="16"/>
       <c r="H17" s="16"/>
       <c r="I17" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="18" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J17" s="33" t="e">
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B18" s="20"/>
+      <c r="B18" s="34" t="s">
+        <v>20</v>
+      </c>
       <c r="C18" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D18" s="16"/>
       <c r="E18" s="16"/>
@@ -2139,18 +2132,18 @@
       <c r="G18" s="16"/>
       <c r="H18" s="16"/>
       <c r="I18" s="17">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="J18" s="21" t="e">
-        <f t="shared" si="4"/>
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J18" s="18" t="e">
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B19" s="22"/>
+      <c r="B19" s="35"/>
       <c r="C19" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D19" s="16"/>
       <c r="E19" s="16"/>
@@ -2158,141 +2151,141 @@
       <c r="G19" s="16"/>
       <c r="H19" s="16"/>
       <c r="I19" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J19" s="20" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B20" s="21"/>
+      <c r="C20" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="F20" s="16"/>
+      <c r="G20" s="16"/>
+      <c r="H20" s="16"/>
+      <c r="I20" s="17">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J20" s="18" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B21" s="36"/>
+      <c r="C21" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="23">
+        <f t="shared" ref="D21:I21" si="3">SUM(D16:D20)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="24">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="J19" s="18" t="e">
-        <f t="shared" si="4"/>
+      <c r="F21" s="25">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="26">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="H21" s="27">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="28">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="J21" s="29" t="e">
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="20" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B20" s="38"/>
-      <c r="C20" s="24" t="s">
+    <row r="22" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="D22" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="31" t="e">
+        <f>(D21+E21)/(I21-F21)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H22" s="31"/>
+      <c r="I22" s="31"/>
+    </row>
+    <row r="23" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="D23" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
+      <c r="G23" s="29" t="e">
+        <f>D21/(I21-F21)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+    </row>
+    <row r="25" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B25" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B26" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I26" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="25">
-        <f t="shared" ref="D20:I20" si="5">SUM(D15:D19)</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="26">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="F20" s="27">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="G20" s="28">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="H20" s="29">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="I20" s="30">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J20" s="31" t="e">
-        <f t="shared" si="4"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="21" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="D21" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="33" t="e">
-        <f>(D20+E20)/(I20-F20)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H21" s="33"/>
-      <c r="I21" s="33"/>
-    </row>
-    <row r="22" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="D22" s="34" t="s">
-        <v>16</v>
-      </c>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="35" t="e">
-        <f>D20/(I20-F20)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-    </row>
-    <row r="24" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B24" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-    </row>
-    <row r="25" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B25" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="F25" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="G25" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="I25" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="J25" s="12" t="s">
+      <c r="J26" s="12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="26" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B26" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C26" s="15" t="s">
+    <row r="27" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B27" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C27" s="15" t="s">
         <v>11</v>
-      </c>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
-      <c r="G26" s="16"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="17">
-        <f t="shared" ref="I26:I29" si="6">SUM(D26:H26)</f>
-        <v>0</v>
-      </c>
-      <c r="J26" s="18" t="e">
-        <f t="shared" ref="J26:J30" si="7">D26/(I26-F26)</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="27" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B27" s="20"/>
-      <c r="C27" s="15" t="s">
-        <v>12</v>
       </c>
       <c r="D27" s="16"/>
       <c r="E27" s="16"/>
@@ -2300,18 +2293,18 @@
       <c r="G27" s="16"/>
       <c r="H27" s="16"/>
       <c r="I27" s="17">
-        <f t="shared" si="6"/>
+        <f>SUM(D27:H27)</f>
         <v>0</v>
       </c>
       <c r="J27" s="18" t="e">
-        <f t="shared" si="7"/>
+        <f>D27/(I27-F27)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="28" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B28" s="20"/>
+      <c r="B28" s="35"/>
       <c r="C28" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
@@ -2319,18 +2312,18 @@
       <c r="G28" s="16"/>
       <c r="H28" s="16"/>
       <c r="I28" s="17">
-        <f t="shared" si="6"/>
+        <f>SUM(D28:H28)</f>
         <v>0</v>
       </c>
       <c r="J28" s="18" t="e">
-        <f t="shared" si="7"/>
+        <f>D28/(I28-F28)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="29" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B29" s="22"/>
+      <c r="B29" s="35"/>
       <c r="C29" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -2338,446 +2331,482 @@
       <c r="G29" s="16"/>
       <c r="H29" s="16"/>
       <c r="I29" s="17">
-        <f t="shared" si="6"/>
+        <f>SUM(D29:H29)</f>
         <v>0</v>
       </c>
       <c r="J29" s="18" t="e">
-        <f t="shared" si="7"/>
+        <f>D29/(I29-F29)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="30" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="B30" s="38"/>
-      <c r="C30" s="24" t="s">
+      <c r="B30" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="16"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="18"/>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B31" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="16"/>
+      <c r="H31" s="16"/>
+      <c r="I31" s="17">
+        <f>SUM(D31:H31)</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="18" t="e">
+        <f>D31/(I31-F31)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="32" s="1" customFormat="1" ht="15.6" spans="2:10">
+      <c r="B32" s="36"/>
+      <c r="C32" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="D30" s="25">
-        <f t="shared" ref="D30:H30" si="8">SUM(D26:D29)</f>
-        <v>0</v>
-      </c>
-      <c r="E30" s="26">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="F30" s="27">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="G30" s="28">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="H30" s="29">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="I30" s="30">
-        <f>SUM(I26:I28)</f>
-        <v>0</v>
-      </c>
-      <c r="J30" s="31" t="e">
-        <f t="shared" si="7"/>
+      <c r="D32" s="23">
+        <f>SUM(D27:D31)</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="24">
+        <f>SUM(E27:E31)</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="25">
+        <f>SUM(F27:F31)</f>
+        <v>0</v>
+      </c>
+      <c r="G32" s="26">
+        <f>SUM(G27:G31)</f>
+        <v>0</v>
+      </c>
+      <c r="H32" s="27">
+        <f>SUM(H27:H31)</f>
+        <v>0</v>
+      </c>
+      <c r="I32" s="28">
+        <f>SUM(I27:I29)</f>
+        <v>0</v>
+      </c>
+      <c r="J32" s="29" t="e">
+        <f>D32/(I32-F32)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="31" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="D31" s="32" t="s">
-        <v>15</v>
-      </c>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="33" t="e">
-        <f>(D30+E30)/(I30-F30)</f>
+    <row r="33" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="D33" s="30" t="s">
+        <v>17</v>
+      </c>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="31" t="e">
+        <f>(D32+E32)/(I32-F32)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H31" s="33"/>
-      <c r="I31" s="33"/>
-    </row>
-    <row r="32" s="1" customFormat="1" ht="15.6" spans="2:10">
-      <c r="D32" s="34" t="s">
-        <v>16</v>
-      </c>
-      <c r="E32" s="34"/>
-      <c r="F32" s="34"/>
-      <c r="G32" s="35" t="e">
-        <f>D30/(I30-F30)</f>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
+    </row>
+    <row r="34" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="D34" s="32" t="s">
+        <v>18</v>
+      </c>
+      <c r="E34" s="32"/>
+      <c r="F34" s="32"/>
+      <c r="G34" s="29" t="e">
+        <f>D32/(I32-F32)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H32" s="35"/>
-      <c r="I32" s="35"/>
-    </row>
-    <row r="33" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="D33" s="39"/>
-      <c r="E33" s="39"/>
-      <c r="F33" s="39"/>
-      <c r="G33" s="40"/>
-      <c r="H33" s="40"/>
-      <c r="I33" s="41"/>
-    </row>
-    <row r="34" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="A34" s="1">
+      <c r="H34" s="29"/>
+      <c r="I34" s="29"/>
+    </row>
+    <row r="35" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="D35" s="37"/>
+      <c r="E35" s="37"/>
+      <c r="F35" s="37"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="39"/>
+    </row>
+    <row r="36" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="A36" s="1">
         <v>164</v>
       </c>
-      <c r="B34" s="42"/>
-      <c r="C34" s="43" t="s">
-        <v>23</v>
-      </c>
-      <c r="D34" s="43"/>
-      <c r="E34" s="43"/>
-      <c r="F34" s="43"/>
-      <c r="G34" s="43"/>
-      <c r="H34" s="43"/>
-    </row>
-    <row r="35" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="C35" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="D35" s="34" t="s">
+      <c r="B36" s="40"/>
+      <c r="C36" s="41" t="s">
         <v>25</v>
       </c>
-      <c r="E35" s="45" t="s">
+      <c r="D36" s="41"/>
+      <c r="E36" s="41"/>
+      <c r="F36" s="41"/>
+      <c r="G36" s="41"/>
+      <c r="H36" s="41"/>
+    </row>
+    <row r="37" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C37" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="F35" s="46" t="s">
+      <c r="D37" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="G35" s="47" t="s">
+      <c r="E37" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="H35" s="48" t="s">
+      <c r="F37" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="G37" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="H37" s="46" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="36" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="C36" s="15" t="s">
+    <row r="38" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C38" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="D36" s="49"/>
-      <c r="E36" s="49"/>
-      <c r="F36" s="50"/>
-      <c r="G36" s="50"/>
-      <c r="H36" s="51">
-        <f>SUM(D36:G36)</f>
-        <v>0</v>
-      </c>
-      <c r="I36" s="52"/>
-    </row>
-    <row r="37" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="C37" s="44" t="s">
+      <c r="D38" s="47"/>
+      <c r="E38" s="47"/>
+      <c r="F38" s="48"/>
+      <c r="G38" s="48"/>
+      <c r="H38" s="49">
+        <f>SUM(D38:G38)</f>
+        <v>0</v>
+      </c>
+      <c r="I38" s="50"/>
+    </row>
+    <row r="39" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C39" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="D37" s="53">
-        <f t="shared" ref="D37:G37" si="9">SUM(D36:D36)</f>
-        <v>0</v>
-      </c>
-      <c r="E37" s="53">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="F37" s="54">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="G37" s="54">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="H37" s="55">
-        <f>SUM(D37:G37)</f>
-        <v>0</v>
-      </c>
-      <c r="I37" s="52"/>
-    </row>
-    <row r="38" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="C38" s="56"/>
-      <c r="D38" s="57" t="s">
+      <c r="D39" s="51">
+        <f t="shared" ref="D39:G39" si="4">SUM(D38:D38)</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="51">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="F39" s="52">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="G39" s="52">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="H39" s="53">
+        <f>SUM(D39:G39)</f>
+        <v>0</v>
+      </c>
+      <c r="I39" s="50"/>
+    </row>
+    <row r="40" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="C40" s="54"/>
+      <c r="D40" s="55" t="s">
+        <v>31</v>
+      </c>
+      <c r="E40" s="55"/>
+      <c r="F40" s="56">
+        <v>0</v>
+      </c>
+      <c r="G40" s="56"/>
+      <c r="H40" s="57"/>
+      <c r="I40" s="50"/>
+    </row>
+    <row r="41" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B41" s="58"/>
+      <c r="C41" s="59"/>
+      <c r="D41" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="E41" s="61"/>
+      <c r="F41" s="56">
+        <v>0</v>
+      </c>
+      <c r="G41" s="56"/>
+      <c r="H41" s="50"/>
+      <c r="I41" s="50"/>
+    </row>
+    <row r="42" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B42" s="58"/>
+      <c r="C42" s="58"/>
+      <c r="D42" s="62"/>
+      <c r="E42" s="62"/>
+      <c r="F42" s="63"/>
+      <c r="G42" s="64"/>
+      <c r="I42" s="50"/>
+    </row>
+    <row r="43" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B43" s="40"/>
+      <c r="C43" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="D43" s="41"/>
+      <c r="E43" s="41"/>
+      <c r="F43" s="41"/>
+      <c r="G43" s="41"/>
+      <c r="H43" s="41"/>
+      <c r="I43" s="50"/>
+    </row>
+    <row r="44" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B44" s="37"/>
+      <c r="C44" s="42" t="s">
+        <v>26</v>
+      </c>
+      <c r="D44" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="E44" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="F44" s="44" t="s">
         <v>29</v>
       </c>
-      <c r="E38" s="57"/>
-      <c r="F38" s="58">
-        <v>0</v>
-      </c>
-      <c r="G38" s="58"/>
-      <c r="H38" s="59"/>
-      <c r="I38" s="52"/>
-    </row>
-    <row r="39" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B39" s="60"/>
-      <c r="C39" s="61"/>
-      <c r="D39" s="62" t="s">
+      <c r="G44" s="45" t="s">
         <v>30</v>
       </c>
-      <c r="E39" s="63"/>
-      <c r="F39" s="58">
-        <v>0</v>
-      </c>
-      <c r="G39" s="58"/>
-      <c r="H39" s="52"/>
-      <c r="I39" s="52"/>
-    </row>
-    <row r="40" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B40" s="60"/>
-      <c r="C40" s="60"/>
-      <c r="D40" s="64"/>
-      <c r="E40" s="64"/>
-      <c r="F40" s="65"/>
-      <c r="G40" s="66"/>
-      <c r="I40" s="52"/>
-    </row>
-    <row r="41" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B41" s="42"/>
-      <c r="C41" s="43" t="s">
+      <c r="H44" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="I44" s="50"/>
+    </row>
+    <row r="45" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B45" s="37"/>
+      <c r="C45" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="65"/>
+      <c r="E45" s="65"/>
+      <c r="F45" s="66"/>
+      <c r="G45" s="66"/>
+      <c r="H45" s="67">
+        <f>SUM(D45:G45)</f>
+        <v>0</v>
+      </c>
+      <c r="I45" s="50"/>
+    </row>
+    <row r="46" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B46" s="37"/>
+      <c r="C46" s="42" t="s">
+        <v>8</v>
+      </c>
+      <c r="D46" s="68">
+        <f>SUM(D45:D45)</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="68">
+        <f>SUM(E45:E45)</f>
+        <v>0</v>
+      </c>
+      <c r="F46" s="69">
+        <f>SUM(F45:F45)</f>
+        <v>0</v>
+      </c>
+      <c r="G46" s="70">
+        <f>SUM(G45:G45)</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="71">
+        <f>SUM(D46:G46)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B47" s="72"/>
+      <c r="C47" s="58"/>
+      <c r="D47" s="55" t="s">
         <v>31</v>
       </c>
-      <c r="D41" s="43"/>
-      <c r="E41" s="43"/>
-      <c r="F41" s="43"/>
-      <c r="G41" s="43"/>
-      <c r="H41" s="43"/>
-      <c r="I41" s="52"/>
-    </row>
-    <row r="42" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B42" s="39"/>
-      <c r="C42" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="D42" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="E42" s="45" t="s">
+      <c r="E47" s="55"/>
+      <c r="F47" s="56">
+        <v>0</v>
+      </c>
+      <c r="G47" s="56"/>
+      <c r="H47" s="73"/>
+    </row>
+    <row r="48" s="1" customFormat="1" ht="15.6" spans="1:9">
+      <c r="B48" s="72"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="E48" s="61"/>
+      <c r="F48" s="74">
+        <v>0</v>
+      </c>
+      <c r="G48" s="75"/>
+      <c r="H48" s="73"/>
+    </row>
+    <row r="50" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C50" s="41" t="s">
+        <v>34</v>
+      </c>
+      <c r="D50" s="41"/>
+      <c r="E50" s="41"/>
+      <c r="F50" s="41"/>
+      <c r="G50" s="41"/>
+      <c r="H50" s="41"/>
+    </row>
+    <row r="51" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C51" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="F42" s="46" t="s">
+      <c r="D51" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="G42" s="47" t="s">
+      <c r="E51" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="H42" s="48" t="s">
+      <c r="F51" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="G51" s="45" t="s">
+        <v>30</v>
+      </c>
+      <c r="H51" s="46" t="s">
         <v>8</v>
-      </c>
-      <c r="I42" s="52"/>
-    </row>
-    <row r="43" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B43" s="39"/>
-      <c r="C43" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" s="67"/>
-      <c r="E43" s="67"/>
-      <c r="F43" s="68"/>
-      <c r="G43" s="68"/>
-      <c r="H43" s="69">
-        <f>SUM(D43:G43)</f>
-        <v>0</v>
-      </c>
-      <c r="I43" s="52"/>
-    </row>
-    <row r="44" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B44" s="39"/>
-      <c r="C44" s="44" t="s">
-        <v>8</v>
-      </c>
-      <c r="D44" s="70">
-        <f>SUM(D43:D43)</f>
-        <v>0</v>
-      </c>
-      <c r="E44" s="70">
-        <f>SUM(E43:E43)</f>
-        <v>0</v>
-      </c>
-      <c r="F44" s="71">
-        <f>SUM(F43:F43)</f>
-        <v>0</v>
-      </c>
-      <c r="G44" s="72">
-        <f>SUM(G43:G43)</f>
-        <v>0</v>
-      </c>
-      <c r="H44" s="73">
-        <f>SUM(D44:G44)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B45" s="74"/>
-      <c r="C45" s="60"/>
-      <c r="D45" s="57" t="s">
-        <v>29</v>
-      </c>
-      <c r="E45" s="57"/>
-      <c r="F45" s="58">
-        <v>0</v>
-      </c>
-      <c r="G45" s="58"/>
-      <c r="H45" s="75"/>
-    </row>
-    <row r="46" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="B46" s="74"/>
-      <c r="C46" s="60"/>
-      <c r="D46" s="62" t="s">
-        <v>30</v>
-      </c>
-      <c r="E46" s="63"/>
-      <c r="F46" s="76">
-        <v>0</v>
-      </c>
-      <c r="G46" s="77"/>
-      <c r="H46" s="75"/>
-    </row>
-    <row r="48" s="1" customFormat="1" ht="15.6" spans="1:9">
-      <c r="C48" s="43" t="s">
-        <v>32</v>
-      </c>
-      <c r="D48" s="43"/>
-      <c r="E48" s="43"/>
-      <c r="F48" s="43"/>
-      <c r="G48" s="43"/>
-      <c r="H48" s="43"/>
-    </row>
-    <row r="49" s="1" customFormat="1" ht="15.6" spans="3:8">
-      <c r="C49" s="44" t="s">
-        <v>24</v>
-      </c>
-      <c r="D49" s="34" t="s">
-        <v>25</v>
-      </c>
-      <c r="E49" s="45" t="s">
-        <v>26</v>
-      </c>
-      <c r="F49" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="G49" s="47" t="s">
-        <v>28</v>
-      </c>
-      <c r="H49" s="48" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="50" s="1" customFormat="1" ht="15.6" spans="3:8">
-      <c r="C50" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="D50" s="49"/>
-      <c r="E50" s="49"/>
-      <c r="F50" s="50"/>
-      <c r="G50" s="50"/>
-      <c r="H50" s="51">
-        <f>SUM(D50:G50)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" s="1" customFormat="1" ht="15.6" spans="3:8">
-      <c r="C51" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="D51" s="49"/>
-      <c r="E51" s="49"/>
-      <c r="F51" s="50"/>
-      <c r="G51" s="50"/>
-      <c r="H51" s="51">
-        <f>SUM(D51:G51)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="52" s="1" customFormat="1" ht="15.6" spans="3:8">
       <c r="C52" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" s="47"/>
+      <c r="E52" s="47"/>
+      <c r="F52" s="48"/>
+      <c r="G52" s="48"/>
+      <c r="H52" s="49">
+        <f>SUM(D52:G52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C53" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D53" s="47"/>
+      <c r="E53" s="47"/>
+      <c r="F53" s="48"/>
+      <c r="G53" s="48"/>
+      <c r="H53" s="49">
+        <f>SUM(D53:G53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C54" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D52" s="49"/>
-      <c r="E52" s="49"/>
-      <c r="F52" s="50"/>
-      <c r="G52" s="50"/>
-      <c r="H52" s="51">
-        <f>SUM(D52:G52)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" s="1" customFormat="1" ht="15.6" spans="3:8">
-      <c r="C53" s="44" t="s">
+      <c r="D54" s="47"/>
+      <c r="E54" s="47"/>
+      <c r="F54" s="48"/>
+      <c r="G54" s="48"/>
+      <c r="H54" s="49">
+        <f>SUM(D54:G54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C55" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="D53" s="53">
-        <f>SUM(D50:D52)</f>
-        <v>0</v>
-      </c>
-      <c r="E53" s="53">
-        <f>SUM(E50:E52)</f>
-        <v>0</v>
-      </c>
-      <c r="F53" s="54">
-        <f>SUM(F50:F52)</f>
-        <v>0</v>
-      </c>
-      <c r="G53" s="54">
-        <f>SUM(G50:G52)</f>
-        <v>0</v>
-      </c>
-      <c r="H53" s="55">
-        <f>SUM(H50:H52)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" s="1" customFormat="1" ht="16" customHeight="1" spans="3:8">
-      <c r="C54" s="56"/>
-      <c r="D54" s="57" t="s">
-        <v>29</v>
-      </c>
-      <c r="E54" s="57"/>
-      <c r="F54" s="58">
-        <v>0</v>
-      </c>
-      <c r="G54" s="58"/>
-      <c r="H54" s="59"/>
-    </row>
-    <row r="55" s="1" customFormat="1" ht="15.6" spans="3:8">
-      <c r="C55" s="61"/>
-      <c r="D55" s="62" t="s">
-        <v>30</v>
-      </c>
-      <c r="E55" s="63"/>
-      <c r="F55" s="58">
-        <v>0</v>
-      </c>
-      <c r="G55" s="58"/>
-      <c r="H55" s="52"/>
+      <c r="D55" s="51">
+        <f>SUM(D52:D54)</f>
+        <v>0</v>
+      </c>
+      <c r="E55" s="51">
+        <f>SUM(E52:E54)</f>
+        <v>0</v>
+      </c>
+      <c r="F55" s="52">
+        <f>SUM(F52:F54)</f>
+        <v>0</v>
+      </c>
+      <c r="G55" s="52">
+        <f>SUM(G52:G54)</f>
+        <v>0</v>
+      </c>
+      <c r="H55" s="53">
+        <f>SUM(H52:H54)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" s="1" customFormat="1" ht="16" customHeight="1" spans="3:8">
+      <c r="C56" s="54"/>
+      <c r="D56" s="55" t="s">
+        <v>31</v>
+      </c>
+      <c r="E56" s="55"/>
+      <c r="F56" s="56">
+        <v>0</v>
+      </c>
+      <c r="G56" s="56"/>
+      <c r="H56" s="57"/>
+    </row>
+    <row r="57" s="1" customFormat="1" ht="15.6" spans="3:8">
+      <c r="C57" s="59"/>
+      <c r="D57" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="E57" s="61"/>
+      <c r="F57" s="56">
+        <v>0</v>
+      </c>
+      <c r="G57" s="56"/>
+      <c r="H57" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="33">
     <mergeCell ref="B2:J2"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="G9:I9"/>
     <mergeCell ref="D10:F10"/>
     <mergeCell ref="G10:I10"/>
-    <mergeCell ref="B13:J13"/>
-    <mergeCell ref="D21:F21"/>
-    <mergeCell ref="G21:I21"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="B14:J14"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="G22:I22"/>
-    <mergeCell ref="B24:J24"/>
-    <mergeCell ref="D31:F31"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="D32:F32"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="C48:H48"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="B25:J25"/>
+    <mergeCell ref="D33:F33"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="D34:F34"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="C50:H50"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="B27:B29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>